<commit_message>
Testing more optimal constraints
</commit_message>
<xml_diff>
--- a/backend/app/scheduler/timetable.xlsx
+++ b/backend/app/scheduler/timetable.xlsx
@@ -680,58 +680,42 @@
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>LIT301_T3</t>
-        </is>
-      </c>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>THEO201_T3</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>THEO301_T2</t>
-        </is>
-      </c>
+      <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>LIT101</t>
-        </is>
-      </c>
+      <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>PHI101</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>THEO101</t>
-        </is>
-      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>HIS201_T3</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr">
-        <is>
-          <t>LIT101_T3</t>
-        </is>
-      </c>
+      <c r="AO4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -741,22 +725,22 @@
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>HIS301_T1</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>THEO201_T2</t>
+          <t>LIT201_T2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>LIT201</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>PHI101_T1</t>
@@ -767,53 +751,45 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>PHI201</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>PHI101_T3</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>LIT201_T3</t>
+        </is>
+      </c>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>THEO301</t>
+        </is>
+      </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>LIT101</t>
+          <t>HIS201</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>PHI301_T3</t>
-        </is>
-      </c>
+      <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>THEO201_T3</t>
-        </is>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>PHI101</t>
-        </is>
-      </c>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>THEO101</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>HIS301_T2</t>
-        </is>
-      </c>
+          <t>LIT301</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
@@ -826,13 +802,17 @@
           <t>11:00–12:00</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
         <is>
           <t>PHI301</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HIS101_T2</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -840,46 +820,62 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>HIS301</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr"/>
+          <t>THEO101</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>LIT201</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>HIS301_T1</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>THEO201_T1</t>
-        </is>
-      </c>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>PHI201</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>HIS301_T3</t>
-        </is>
-      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>THEO301_T3</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>THEO301</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>HIS201</t>
+        </is>
+      </c>
       <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>LIT101_T2</t>
+        </is>
+      </c>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>LIT301</t>
+        </is>
+      </c>
       <c r="AJ6" t="inlineStr">
         <is>
           <t>PHI201_T3</t>
@@ -893,7 +889,11 @@
           <t>THEO301_T1</t>
         </is>
       </c>
-      <c r="AO6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>HIS101_T3</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -901,23 +901,19 @@
           <t>12:00–13:00</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
         <is>
           <t>PHI301</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>HIS201_T3</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>LIT301_T2</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LIT101_T1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
@@ -927,22 +923,14 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>HIS301</t>
+          <t>THEO101</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>LIT301_T1</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>PHI201_T1</t>
-        </is>
-      </c>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
@@ -952,30 +940,30 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>THEO101_T3</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>LIT201</t>
-        </is>
-      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>HIS201_T1</t>
-        </is>
-      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>HIS201_T2</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>PHI201</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>HIS301</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
@@ -995,49 +983,69 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>PHI101_T2</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>LIT101</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>HIS201_T2</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>PHI301_T3</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>THEO101_T3</t>
+        </is>
+      </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>PHI101_T2</t>
+        </is>
+      </c>
       <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>LIT201</t>
-        </is>
-      </c>
-      <c r="AA8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>THEO201</t>
+        </is>
+      </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>PHI201</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>HIS301</t>
+        </is>
+      </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>LIT301_T3</t>
+        </is>
+      </c>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
     </row>
@@ -1048,12 +1056,12 @@
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>HIS201</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PHI201_T1</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -1061,7 +1069,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>THEO301</t>
+          <t>LIT101</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
@@ -1069,7 +1077,7 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>LIT201_T2</t>
+          <t>THEO301_T2</t>
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
@@ -1077,39 +1085,35 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>THEO101_T1</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>HIS101_T3</t>
-        </is>
-      </c>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr">
         <is>
-          <t>PHI301_T2</t>
+          <t>LIT101_T3</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>THEO201</t>
+        </is>
+      </c>
       <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>PHI301_T1</t>
         </is>
       </c>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>HIS101_T2</t>
-        </is>
-      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>LIT301_T1</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr"/>
@@ -1117,12 +1121,12 @@
       <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
-      <c r="AN9" t="inlineStr">
-        <is>
-          <t>PHI201_T2</t>
-        </is>
-      </c>
-      <c r="AO9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>HIS101_T1</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1131,63 +1135,59 @@
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>HIS201</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LIT301_T2</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>THEO301_T3</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>THEO201_T2</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>PHI101</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>HIS301_T3</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
         <is>
           <t>LIT201_T1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>THEO301</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>LIT301</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>PHI101_T3</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>THEO201</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>HIS301_T2</t>
+        </is>
+      </c>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PHI301_T2</t>
+        </is>
+      </c>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>HIS101</t>
-        </is>
-      </c>
+      <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
@@ -1195,15 +1195,27 @@
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>LIT101_T2</t>
+          <t>HIS201_T1</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>HIS101</t>
+        </is>
+      </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>PHI201_T2</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>THEO201_T1</t>
+        </is>
+      </c>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
     </row>
@@ -1224,7 +1236,7 @@
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>LIT301</t>
+          <t>PHI101</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1234,31 +1246,19 @@
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>THEO201</t>
-        </is>
-      </c>
+      <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>HIS101_T1</t>
+          <t>THEO101_T1</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>LIT101_T1</t>
-        </is>
-      </c>
+      <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>HIS101</t>
-        </is>
-      </c>
+      <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
@@ -1266,15 +1266,15 @@
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>HIS101</t>
+        </is>
+      </c>
       <c r="AJ11" t="inlineStr"/>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="inlineStr">
-        <is>
-          <t>LIT201_T3</t>
-        </is>
-      </c>
+      <c r="AM11" t="inlineStr"/>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
I thought I already did this lol, optimizing constraints
</commit_message>
<xml_diff>
--- a/backend/app/scheduler/timetable.xlsx
+++ b/backend/app/scheduler/timetable.xlsx
@@ -670,14 +670,22 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>THEO101_T1</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>PHI201</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -686,11 +694,7 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>THEO201_T3</t>
-        </is>
-      </c>
+      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
@@ -703,11 +707,7 @@
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr">
-        <is>
-          <t>HIS201_T3</t>
-        </is>
-      </c>
+      <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
@@ -724,75 +724,83 @@
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HIS201</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>LIT201_T2</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PHI301_T2</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>HIS301</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>LIT201</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>PHI101_T1</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+          <t>PHI201</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>THEO301_T2</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>THEO201</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>PHI101_T3</t>
-        </is>
-      </c>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>LIT201_T3</t>
+          <t>HIS301_T1</t>
         </is>
       </c>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>THEO301</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>HIS201</t>
-        </is>
-      </c>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>HIS101_T3</t>
+        </is>
+      </c>
       <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>LIT301</t>
-        </is>
-      </c>
+      <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>THEO201_T2</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>LIT201_T3</t>
+        </is>
+      </c>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
     </row>
@@ -805,95 +813,75 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PHI301</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>HIS101_T2</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>HIS201</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>THEO101_T3</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>THEO101</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>LIT201</t>
-        </is>
-      </c>
+          <t>HIS301</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>HIS301_T1</t>
-        </is>
-      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>PHI101_T1</t>
+        </is>
+      </c>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>THEO201</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>THEO301_T3</t>
-        </is>
-      </c>
-      <c r="W6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>LIT101_T2</t>
+        </is>
+      </c>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>THEO301</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>HIS201</t>
-        </is>
-      </c>
+          <t>PHI301</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t>LIT101_T2</t>
-        </is>
-      </c>
-      <c r="AD6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>LIT201_T2</t>
+        </is>
+      </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>LIT301</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>PHI201_T3</t>
-        </is>
-      </c>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr">
-        <is>
-          <t>THEO301_T1</t>
-        </is>
-      </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>HIS101_T3</t>
-        </is>
-      </c>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -902,31 +890,27 @@
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>PHI301</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LIT101_T1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>HIS101_T1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LIT301_T1</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>THEO101_T2</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>THEO101</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>LIT201</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
@@ -940,35 +924,51 @@
       <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>HIS201_T3</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>PHI301</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>LIT301</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>THEO201_T1</t>
+        </is>
+      </c>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>HIS201_T2</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>PHI201</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>HIS301</t>
-        </is>
-      </c>
-      <c r="AJ7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>HIS201_T1</t>
+        </is>
+      </c>
       <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>THEO101_T2</t>
+        </is>
+      </c>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>PHI101_T3</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -977,75 +977,83 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>HIS101</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>THEO201_T3</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>LIT101</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>PHI201_T1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>LIT201</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>PHI301_T3</t>
-        </is>
-      </c>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>HIS101_T2</t>
+        </is>
+      </c>
       <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>THEO101_T3</t>
-        </is>
-      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>THEO301</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
       <c r="X8" t="inlineStr">
         <is>
-          <t>PHI101_T2</t>
+          <t>LIT301_T3</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>THEO201</t>
+          <t>LIT301</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>HIS301_T2</t>
+        </is>
+      </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>PHI201</t>
-        </is>
-      </c>
-      <c r="AI8" t="inlineStr">
-        <is>
-          <t>HIS301</t>
-        </is>
-      </c>
-      <c r="AJ8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>LIT201_T1</t>
+        </is>
+      </c>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr">
-        <is>
-          <t>LIT301_T3</t>
-        </is>
-      </c>
+      <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
     </row>
@@ -1056,77 +1064,73 @@
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>PHI201_T1</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>HIS101</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>LIT101</t>
-        </is>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>THEO301_T2</t>
+          <t>PHI101_T2</t>
         </is>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>THEO301</t>
+        </is>
+      </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>LIT101_T3</t>
-        </is>
-      </c>
+      <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t>THEO201</t>
-        </is>
-      </c>
+      <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
-      <c r="AC9" t="inlineStr">
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>THEO301_T1</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>LIT101</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>HIS301_T3</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr">
         <is>
           <t>PHI301_T1</t>
         </is>
       </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t>LIT301_T1</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
-      <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>HIS101_T1</t>
-        </is>
-      </c>
+      <c r="AO9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1134,88 +1138,76 @@
           <t>15:00–16:00</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>THEO101</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PHI201_T2</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>LIT301_T2</t>
+          <t>LIT101_T1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>THEO201_T2</t>
-        </is>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>PHI101</t>
-        </is>
-      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>HIS301_T3</t>
+          <t>HIS201_T2</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>LIT201_T1</t>
-        </is>
-      </c>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>HIS301_T2</t>
-        </is>
-      </c>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>PHI301_T2</t>
+          <t>PHI301_T3</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
-      <c r="AB10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>PHI101</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>LIT101_T3</t>
+        </is>
+      </c>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>HIS201_T1</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>HIS101</t>
-        </is>
-      </c>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>LIT101</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
-      <c r="AL10" t="inlineStr">
-        <is>
-          <t>PHI201_T2</t>
-        </is>
-      </c>
-      <c r="AM10" t="inlineStr">
-        <is>
-          <t>THEO201_T1</t>
-        </is>
-      </c>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
     </row>
@@ -1225,7 +1217,11 @@
           <t>16:00–17:00</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>THEO101</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
@@ -1234,31 +1230,35 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>PHI101</t>
-        </is>
-      </c>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>LIT301_T2</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>THEO101_T1</t>
-        </is>
-      </c>
+      <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>THEO301_T3</t>
+        </is>
+      </c>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>PHI101</t>
+        </is>
+      </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
@@ -1266,12 +1266,12 @@
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr">
-        <is>
-          <t>HIS101</t>
-        </is>
-      </c>
-      <c r="AJ11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>PHI201_T3</t>
+        </is>
+      </c>
       <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="inlineStr"/>

</xml_diff>

<commit_message>
Added SC1 and fixed bug in LC1
</commit_message>
<xml_diff>
--- a/backend/app/scheduler/timetable.xlsx
+++ b/backend/app/scheduler/timetable.xlsx
@@ -670,48 +670,76 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>THEO101_T1</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>LIT101_T2</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>PHI201</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>THEO201_T3</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>HIS301</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>THEO101_T2</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>THEO101</t>
+        </is>
+      </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>PHI301_T3</t>
+        </is>
+      </c>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>HIS301_T3</t>
+        </is>
+      </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>PHI301</t>
+        </is>
+      </c>
       <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>LIT201_T2</t>
+        </is>
+      </c>
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr"/>
@@ -724,55 +752,43 @@
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>HIS201</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PHI101_T1</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>PHI301_T2</t>
-        </is>
-      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>HIS301</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>PHI201</t>
-        </is>
-      </c>
+      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>THEO301_T2</t>
-        </is>
-      </c>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>THEO201</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>THEO101</t>
+        </is>
+      </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>HIS301_T1</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>HIS201_T2</t>
+        </is>
+      </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
@@ -781,26 +797,22 @@
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>HIS101_T3</t>
-        </is>
-      </c>
-      <c r="AG5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>PHI201_T3</t>
+        </is>
+      </c>
       <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>PHI301</t>
+        </is>
+      </c>
       <c r="AJ5" t="inlineStr"/>
       <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>THEO201_T2</t>
-        </is>
-      </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>LIT201_T3</t>
-        </is>
-      </c>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr"/>
       <c r="AO5" t="inlineStr"/>
     </row>
@@ -813,64 +825,48 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>HIS201</t>
+          <t>THEO301</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>THEO101_T3</t>
-        </is>
-      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>HIS201_T3</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>HIS301</t>
-        </is>
-      </c>
+      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>HIS101_T2</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>PHI101_T1</t>
+          <t>LIT201_T3</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>THEO201</t>
-        </is>
-      </c>
+      <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr">
-        <is>
-          <t>LIT101_T2</t>
-        </is>
-      </c>
+      <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>PHI301</t>
-        </is>
-      </c>
+      <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>LIT201_T2</t>
-        </is>
-      </c>
+      <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
@@ -890,15 +886,15 @@
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>HIS101_T1</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>THEO301</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LIT301_T1</t>
+          <t>PHI101_T2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -906,67 +902,67 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>LIT201</t>
-        </is>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>THEO301_T2</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>PHI201</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>THEO101_T3</t>
+        </is>
+      </c>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>LIT301_T1</t>
+        </is>
+      </c>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>HIS201_T3</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>PHI301</t>
-        </is>
-      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>LIT301</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>THEO201_T1</t>
-        </is>
-      </c>
+          <t>HIS201</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>THEO301_T3</t>
+        </is>
+      </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
       <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>HIS201_T1</t>
-        </is>
-      </c>
+      <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="inlineStr">
         <is>
-          <t>THEO101_T2</t>
+          <t>HIS101_T1</t>
         </is>
       </c>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>PHI101_T3</t>
+          <t>LIT301_T2</t>
         </is>
       </c>
     </row>
@@ -977,80 +973,68 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>HIS101</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>THEO201_T3</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>PHI201_T1</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>THEO201_T1</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>HIS301_T2</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>LIT201</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>LIT101_T3</t>
+        </is>
+      </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>HIS101_T3</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>HIS101_T2</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>THEO301</t>
-        </is>
-      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>PHI201</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>LIT301_T3</t>
-        </is>
-      </c>
+      <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>LIT301</t>
+          <t>HIS201</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr">
-        <is>
-          <t>HIS301_T2</t>
-        </is>
-      </c>
-      <c r="AF8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>PHI101_T3</t>
+        </is>
+      </c>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr">
-        <is>
-          <t>LIT201_T1</t>
-        </is>
-      </c>
+      <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr"/>
@@ -1064,11 +1048,7 @@
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>HIS101</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
@@ -1078,25 +1058,29 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>PHI101_T2</t>
-        </is>
-      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>PHI201_T1</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr">
         <is>
-          <t>THEO301</t>
+          <t>HIS101</t>
         </is>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr"/>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>THEO201_T2</t>
+        </is>
+      </c>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
@@ -1105,29 +1089,25 @@
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr">
-        <is>
-          <t>THEO301_T1</t>
-        </is>
-      </c>
+      <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>LIT101</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr"/>
+          <t>THEO201</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>PHI101</t>
+        </is>
+      </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>HIS301_T3</t>
+          <t>LIT301_T3</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr"/>
-      <c r="AL9" t="inlineStr">
-        <is>
-          <t>PHI301_T1</t>
-        </is>
-      </c>
+      <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr"/>
@@ -1140,70 +1120,78 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>THEO101</t>
+          <t>LIT301</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>PHI201_T2</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>LIT101_T1</t>
-        </is>
-      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>HIS201_T1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>LIT101</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>HIS201_T2</t>
+          <t>HIS301_T1</t>
         </is>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>HIS101</t>
+        </is>
+      </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>PHI301_T3</t>
+          <t>PHI301_T2</t>
         </is>
       </c>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>PHI101</t>
-        </is>
-      </c>
-      <c r="AB10" t="inlineStr">
-        <is>
-          <t>LIT101_T3</t>
-        </is>
-      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>LIT201</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>THEO301_T1</t>
+        </is>
+      </c>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>LIT101</t>
-        </is>
-      </c>
-      <c r="AI10" t="inlineStr"/>
+          <t>THEO201</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>PHI101</t>
+        </is>
+      </c>
       <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="inlineStr"/>
@@ -1219,46 +1207,54 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>THEO101</t>
+          <t>LIT301</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>THEO101_T1</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>LIT101</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>LIT301_T2</t>
-        </is>
-      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>PHI201_T2</t>
+        </is>
+      </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>THEO301_T3</t>
-        </is>
-      </c>
+      <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr">
-        <is>
-          <t>PHI101</t>
-        </is>
-      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>LIT101_T1</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>LIT201</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
@@ -1267,14 +1263,18 @@
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr">
-        <is>
-          <t>PHI201_T3</t>
-        </is>
-      </c>
-      <c r="AK11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>LIT201_T1</t>
+        </is>
+      </c>
       <c r="AL11" t="inlineStr"/>
-      <c r="AM11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>PHI301_T1</t>
+        </is>
+      </c>
       <c r="AN11" t="inlineStr"/>
       <c r="AO11" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
FastAPI for backend logic, crude frontend added
</commit_message>
<xml_diff>
--- a/backend/app/scheduler/timetable.xlsx
+++ b/backend/app/scheduler/timetable.xlsx
@@ -670,52 +670,48 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>THEO101_T2</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>LIT101_T2</t>
-        </is>
-      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>THEO201_T3</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>HIS301</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>HIS201_T3</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>THEO101_T2</t>
-        </is>
-      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>THEO101</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>PHI101</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>THEO201_T1</t>
+        </is>
+      </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>PHI301_T3</t>
-        </is>
-      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>LIT301_T1</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
@@ -723,26 +719,30 @@
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>HIS301_T3</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr"/>
+          <t>LIT101_T1</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>THEO201_T2</t>
+        </is>
+      </c>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>PHI301</t>
+          <t>LIT201</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>LIT201_T2</t>
-        </is>
-      </c>
+      <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>HIS301_T2</t>
+        </is>
+      </c>
       <c r="AO4" t="inlineStr"/>
     </row>
     <row r="5">
@@ -755,40 +755,36 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>PHI101_T1</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>LIT301_T3</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>HIS301</t>
-        </is>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>THEO201_T3</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>THEO101</t>
-        </is>
-      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>PHI101</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>HIS201_T2</t>
-        </is>
-      </c>
+      <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
@@ -797,16 +793,16 @@
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr">
-        <is>
-          <t>PHI201_T3</t>
-        </is>
-      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>HIS301_T1</t>
+        </is>
+      </c>
+      <c r="AG5" t="inlineStr"/>
       <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>PHI301</t>
+          <t>LIT201</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr"/>
@@ -823,38 +819,34 @@
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>THEO301</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>HIS201_T3</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>HIS101_T3</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>HIS101_T2</t>
-        </is>
-      </c>
+      <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>LIT201_T3</t>
-        </is>
-      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>PHI301_T3</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>PHI201</t>
+        </is>
+      </c>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -864,20 +856,36 @@
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>PHI101_T3</t>
+        </is>
+      </c>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>LIT301</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>THEO101</t>
+        </is>
+      </c>
       <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>PHI201_T2</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -886,31 +894,27 @@
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>THEO301</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PHI101_T2</t>
+          <t>THEO301_T3</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HIS101</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>THEO301_T2</t>
-        </is>
-      </c>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
@@ -919,52 +923,48 @@
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>THEO101_T3</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>LIT301_T1</t>
-        </is>
-      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>THEO301_T1</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>HIS201</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>HIS301</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>LIT201_T1</t>
+        </is>
+      </c>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>THEO301_T3</t>
-        </is>
-      </c>
+      <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>LIT301</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>THEO101</t>
+        </is>
+      </c>
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>HIS101_T1</t>
-        </is>
-      </c>
+      <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>LIT301_T2</t>
-        </is>
-      </c>
+      <c r="AO7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -976,66 +976,74 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>THEO201_T1</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>HIS301_T2</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HIS101</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>LIT101_T3</t>
-        </is>
-      </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>HIS101_T3</t>
-        </is>
-      </c>
+      <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>PHI201</t>
-        </is>
-      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>THEO301_T2</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>PHI101_T2</t>
+        </is>
+      </c>
       <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr">
-        <is>
-          <t>HIS201</t>
-        </is>
-      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>LIT201_T2</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>HIS301</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>PHI101_T1</t>
+        </is>
+      </c>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="inlineStr"/>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>PHI101_T3</t>
-        </is>
-      </c>
+      <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>LIT101</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>HIS201</t>
+        </is>
+      </c>
       <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>PHI301_T2</t>
+        </is>
+      </c>
       <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
@@ -1049,7 +1057,11 @@
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>THEO101_T1</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -1058,29 +1070,21 @@
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr">
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
         <is>
           <t>PHI201_T1</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>HIS101</t>
-        </is>
-      </c>
+      <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="inlineStr"/>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>THEO201_T2</t>
-        </is>
-      </c>
+      <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr"/>
@@ -1089,23 +1093,23 @@
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="inlineStr"/>
-      <c r="AF9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>HIS301_T3</t>
+        </is>
+      </c>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>THEO201</t>
+          <t>LIT101</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>PHI101</t>
-        </is>
-      </c>
-      <c r="AJ9" t="inlineStr">
-        <is>
-          <t>LIT301_T3</t>
-        </is>
-      </c>
+          <t>HIS201</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="inlineStr"/>
@@ -1118,84 +1122,76 @@
           <t>15:00–16:00</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>LIT301</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PHI301</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LIT201_T3</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>HIS201_T1</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>LIT101</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>THEO301</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>HIS301_T1</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>LIT101_T3</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
-          <t>HIS101</t>
+          <t>THEO201</t>
         </is>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>PHI301_T2</t>
-        </is>
-      </c>
+      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>LIT201</t>
-        </is>
-      </c>
+      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr">
-        <is>
-          <t>THEO301_T1</t>
-        </is>
-      </c>
+      <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
-      <c r="AG10" t="inlineStr"/>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>THEO201</t>
-        </is>
-      </c>
-      <c r="AI10" t="inlineStr">
-        <is>
-          <t>PHI101</t>
-        </is>
-      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>PHI301_T1</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
       <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>LIT301_T2</t>
+        </is>
+      </c>
       <c r="AL10" t="inlineStr"/>
-      <c r="AM10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>PHI201_T3</t>
+        </is>
+      </c>
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr"/>
     </row>
@@ -1205,74 +1201,78 @@
           <t>16:00–17:00</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>LIT301</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>THEO101_T1</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PHI301</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>THEO101_T3</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>LIT101</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>THEO301</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>PHI201_T2</t>
-        </is>
-      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>HIS201_T1</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>THEO201</t>
+        </is>
+      </c>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>LIT101_T1</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>LIT201</t>
-        </is>
-      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>HIS101_T2</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
-      <c r="AC11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>HIS201_T2</t>
+        </is>
+      </c>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
-      <c r="AF11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>LIT101_T2</t>
+        </is>
+      </c>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr"/>
       <c r="AI11" t="inlineStr"/>
       <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr">
-        <is>
-          <t>LIT201_T1</t>
-        </is>
-      </c>
+      <c r="AK11" t="inlineStr"/>
       <c r="AL11" t="inlineStr"/>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>PHI301_T1</t>
+          <t>HIS101_T1</t>
         </is>
       </c>
       <c r="AN11" t="inlineStr"/>

</xml_diff>